<commit_message>
072525 - updated week 12 skins
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Weekly Stats - Week 12.xlsx
+++ b/public/results/2025/2025 Weekly Stats - Week 12.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD239960-DFDC-1344-A761-9FE852991918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EB05767-DC91-474C-AA4B-A226B50DCCF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="44200" yWindow="2000" windowWidth="26740" windowHeight="18000" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -416,7 +416,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -598,18 +598,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -8615,34 +8603,34 @@
         <v>34</v>
       </c>
       <c r="B9" s="12"/>
-      <c r="C9" s="68">
-        <v>6</v>
-      </c>
-      <c r="D9" s="68">
-        <v>5</v>
-      </c>
-      <c r="E9" s="68">
-        <v>5</v>
-      </c>
-      <c r="F9" s="68">
-        <v>4</v>
-      </c>
-      <c r="G9" s="68">
-        <v>6</v>
-      </c>
-      <c r="H9" s="68">
-        <v>4</v>
-      </c>
-      <c r="I9" s="68">
-        <v>3</v>
-      </c>
-      <c r="J9" s="68">
-        <v>5</v>
-      </c>
-      <c r="K9" s="68">
-        <v>6</v>
-      </c>
-      <c r="L9" s="69">
+      <c r="C9" s="12">
+        <v>6</v>
+      </c>
+      <c r="D9" s="12">
+        <v>5</v>
+      </c>
+      <c r="E9" s="12">
+        <v>5</v>
+      </c>
+      <c r="F9" s="12">
+        <v>4</v>
+      </c>
+      <c r="G9" s="12">
+        <v>6</v>
+      </c>
+      <c r="H9" s="12">
+        <v>4</v>
+      </c>
+      <c r="I9" s="12">
+        <v>3</v>
+      </c>
+      <c r="J9" s="12">
+        <v>5</v>
+      </c>
+      <c r="K9" s="12">
+        <v>6</v>
+      </c>
+      <c r="L9" s="13">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
@@ -8669,43 +8657,43 @@
     <row r="10" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15"/>
       <c r="B10" s="16"/>
-      <c r="C10" s="70">
+      <c r="C10" s="16">
         <f>IF(C9&gt;0, VLOOKUP(C9-C$5-(INT($M9/9)+(MOD($M9,9)&gt;=C$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="D10" s="70">
+      <c r="D10" s="16">
         <f>IF(D9&gt;0, VLOOKUP(D9-D$5-(INT($M9/9)+(MOD($M9,9)&gt;=D$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="E10" s="70">
+      <c r="E10" s="16">
         <f>IF(E9&gt;0, VLOOKUP(E9-E$5-(INT($M9/9)+(MOD($M9,9)&gt;=E$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="F10" s="70">
+      <c r="F10" s="16">
         <f>IF(F9&gt;0, VLOOKUP(F9-F$5-(INT($M9/9)+(MOD($M9,9)&gt;=F$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="G10" s="70">
+      <c r="G10" s="16">
         <f>IF(G9&gt;0, VLOOKUP(G9-G$5-(INT($M9/9)+(MOD($M9,9)&gt;=G$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="H10" s="70">
+      <c r="H10" s="16">
         <f>IF(H9&gt;0, VLOOKUP(H9-H$5-(INT($M9/9)+(MOD($M9,9)&gt;=H$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="I10" s="70">
+      <c r="I10" s="16">
         <f>IF(I9&gt;0, VLOOKUP(I9-I$5-(INT($M9/9)+(MOD($M9,9)&gt;=I$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="J10" s="70">
+      <c r="J10" s="16">
         <f>IF(J9&gt;0, VLOOKUP(J9-J$5-(INT($M9/9)+(MOD($M9,9)&gt;=J$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="K10" s="70">
+      <c r="K10" s="16">
         <f>IF(K9&gt;0, VLOOKUP(K9-K$5-(INT($M9/9)+(MOD($M9,9)&gt;=K$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="L10" s="71">
+      <c r="L10" s="17">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
@@ -8732,34 +8720,34 @@
         <v>33</v>
       </c>
       <c r="B11" s="12"/>
-      <c r="C11" s="68">
-        <v>5</v>
-      </c>
-      <c r="D11" s="68">
+      <c r="C11" s="12">
+        <v>5</v>
+      </c>
+      <c r="D11" s="12">
         <v>7</v>
       </c>
-      <c r="E11" s="68">
-        <v>5</v>
-      </c>
-      <c r="F11" s="68">
-        <v>4</v>
-      </c>
-      <c r="G11" s="68">
-        <v>6</v>
-      </c>
-      <c r="H11" s="68">
-        <v>5</v>
-      </c>
-      <c r="I11" s="68">
-        <v>3</v>
-      </c>
-      <c r="J11" s="68">
-        <v>5</v>
-      </c>
-      <c r="K11" s="68">
+      <c r="E11" s="12">
+        <v>5</v>
+      </c>
+      <c r="F11" s="12">
+        <v>4</v>
+      </c>
+      <c r="G11" s="12">
+        <v>6</v>
+      </c>
+      <c r="H11" s="12">
+        <v>5</v>
+      </c>
+      <c r="I11" s="12">
+        <v>3</v>
+      </c>
+      <c r="J11" s="12">
+        <v>5</v>
+      </c>
+      <c r="K11" s="12">
         <v>7</v>
       </c>
-      <c r="L11" s="69">
+      <c r="L11" s="13">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
@@ -8786,43 +8774,43 @@
     <row r="12" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="15"/>
       <c r="B12" s="16"/>
-      <c r="C12" s="70">
+      <c r="C12" s="16">
         <f>IF(C11&gt;0, VLOOKUP(C11-C$5-(INT($M11/9)+(MOD($M11,9)&gt;=C$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="D12" s="70">
+      <c r="D12" s="16">
         <f>IF(D11&gt;0, VLOOKUP(D11-D$5-(INT($M11/9)+(MOD($M11,9)&gt;=D$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="E12" s="70">
+      <c r="E12" s="16">
         <f>IF(E11&gt;0, VLOOKUP(E11-E$5-(INT($M11/9)+(MOD($M11,9)&gt;=E$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="F12" s="70">
+      <c r="F12" s="16">
         <f>IF(F11&gt;0, VLOOKUP(F11-F$5-(INT($M11/9)+(MOD($M11,9)&gt;=F$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="G12" s="70">
+      <c r="G12" s="16">
         <f>IF(G11&gt;0, VLOOKUP(G11-G$5-(INT($M11/9)+(MOD($M11,9)&gt;=G$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="H12" s="70">
+      <c r="H12" s="16">
         <f>IF(H11&gt;0, VLOOKUP(H11-H$5-(INT($M11/9)+(MOD($M11,9)&gt;=H$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="I12" s="70">
+      <c r="I12" s="16">
         <f>IF(I11&gt;0, VLOOKUP(I11-I$5-(INT($M11/9)+(MOD($M11,9)&gt;=I$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="J12" s="70">
+      <c r="J12" s="16">
         <f>IF(J11&gt;0, VLOOKUP(J11-J$5-(INT($M11/9)+(MOD($M11,9)&gt;=J$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="K12" s="70">
+      <c r="K12" s="16">
         <f>IF(K11&gt;0, VLOOKUP(K11-K$5-(INT($M11/9)+(MOD($M11,9)&gt;=K$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="L12" s="71">
+      <c r="L12" s="17">
         <f t="shared" ref="L12" si="1">IF(SUM(C12:K12)&gt;0, SUM(C12:K12),"")</f>
         <v>16</v>
       </c>
@@ -8849,34 +8837,34 @@
         <v>29</v>
       </c>
       <c r="B13" s="12"/>
-      <c r="C13" s="68">
-        <v>5</v>
-      </c>
-      <c r="D13" s="68">
+      <c r="C13" s="12">
+        <v>5</v>
+      </c>
+      <c r="D13" s="12">
         <v>7</v>
       </c>
-      <c r="E13" s="68">
-        <v>5</v>
-      </c>
-      <c r="F13" s="68">
-        <v>5</v>
-      </c>
-      <c r="G13" s="68">
-        <v>6</v>
-      </c>
-      <c r="H13" s="68">
-        <v>5</v>
-      </c>
-      <c r="I13" s="68">
-        <v>4</v>
-      </c>
-      <c r="J13" s="68">
-        <v>6</v>
-      </c>
-      <c r="K13" s="68">
+      <c r="E13" s="12">
+        <v>5</v>
+      </c>
+      <c r="F13" s="12">
+        <v>5</v>
+      </c>
+      <c r="G13" s="12">
+        <v>6</v>
+      </c>
+      <c r="H13" s="12">
+        <v>5</v>
+      </c>
+      <c r="I13" s="12">
+        <v>4</v>
+      </c>
+      <c r="J13" s="12">
+        <v>6</v>
+      </c>
+      <c r="K13" s="12">
         <v>7</v>
       </c>
-      <c r="L13" s="69">
+      <c r="L13" s="13">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
@@ -8903,43 +8891,43 @@
     <row r="14" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15"/>
       <c r="B14" s="16"/>
-      <c r="C14" s="70">
+      <c r="C14" s="16">
         <f>IF(C13&gt;0, VLOOKUP(C13-C$5-(INT($M13/9)+(MOD($M13,9)&gt;=C$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="D14" s="70">
+      <c r="D14" s="16">
         <f>IF(D13&gt;0, VLOOKUP(D13-D$5-(INT($M13/9)+(MOD($M13,9)&gt;=D$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="E14" s="70">
+      <c r="E14" s="16">
         <f>IF(E13&gt;0, VLOOKUP(E13-E$5-(INT($M13/9)+(MOD($M13,9)&gt;=E$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="F14" s="70">
+      <c r="F14" s="16">
         <f>IF(F13&gt;0, VLOOKUP(F13-F$5-(INT($M13/9)+(MOD($M13,9)&gt;=F$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="G14" s="70">
+      <c r="G14" s="16">
         <f>IF(G13&gt;0, VLOOKUP(G13-G$5-(INT($M13/9)+(MOD($M13,9)&gt;=G$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="H14" s="70">
+      <c r="H14" s="16">
         <f>IF(H13&gt;0, VLOOKUP(H13-H$5-(INT($M13/9)+(MOD($M13,9)&gt;=H$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="I14" s="70">
+      <c r="I14" s="16">
         <f>IF(I13&gt;0, VLOOKUP(I13-I$5-(INT($M13/9)+(MOD($M13,9)&gt;=I$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="J14" s="70">
+      <c r="J14" s="16">
         <f>IF(J13&gt;0, VLOOKUP(J13-J$5-(INT($M13/9)+(MOD($M13,9)&gt;=J$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="K14" s="70">
+      <c r="K14" s="16">
         <f>IF(K13&gt;0, VLOOKUP(K13-K$5-(INT($M13/9)+(MOD($M13,9)&gt;=K$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="L14" s="71">
+      <c r="L14" s="17">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
@@ -8966,34 +8954,34 @@
         <v>14</v>
       </c>
       <c r="B15" s="12"/>
-      <c r="C15" s="68">
-        <v>5</v>
-      </c>
-      <c r="D15" s="68">
+      <c r="C15" s="12">
+        <v>5</v>
+      </c>
+      <c r="D15" s="12">
         <v>7</v>
       </c>
-      <c r="E15" s="68">
-        <v>5</v>
-      </c>
-      <c r="F15" s="68">
-        <v>5</v>
-      </c>
-      <c r="G15" s="68">
-        <v>6</v>
-      </c>
-      <c r="H15" s="68">
+      <c r="E15" s="12">
+        <v>5</v>
+      </c>
+      <c r="F15" s="12">
+        <v>5</v>
+      </c>
+      <c r="G15" s="12">
+        <v>6</v>
+      </c>
+      <c r="H15" s="12">
         <v>7</v>
       </c>
-      <c r="I15" s="68">
-        <v>5</v>
-      </c>
-      <c r="J15" s="68">
-        <v>5</v>
-      </c>
-      <c r="K15" s="68">
+      <c r="I15" s="12">
+        <v>5</v>
+      </c>
+      <c r="J15" s="12">
+        <v>5</v>
+      </c>
+      <c r="K15" s="12">
         <v>7</v>
       </c>
-      <c r="L15" s="69">
+      <c r="L15" s="13">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
@@ -9020,43 +9008,43 @@
     <row r="16" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="15"/>
       <c r="B16" s="16"/>
-      <c r="C16" s="70">
+      <c r="C16" s="16">
         <f>IF(C15&gt;0, VLOOKUP(C15-C$5-(INT($M15/9)+(MOD($M15,9)&gt;=C$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="D16" s="70">
+      <c r="D16" s="16">
         <f>IF(D15&gt;0, VLOOKUP(D15-D$5-(INT($M15/9)+(MOD($M15,9)&gt;=D$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="E16" s="70">
+      <c r="E16" s="16">
         <f>IF(E15&gt;0, VLOOKUP(E15-E$5-(INT($M15/9)+(MOD($M15,9)&gt;=E$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="F16" s="70">
+      <c r="F16" s="16">
         <f>IF(F15&gt;0, VLOOKUP(F15-F$5-(INT($M15/9)+(MOD($M15,9)&gt;=F$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="G16" s="70">
+      <c r="G16" s="16">
         <f>IF(G15&gt;0, VLOOKUP(G15-G$5-(INT($M15/9)+(MOD($M15,9)&gt;=G$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="H16" s="70">
+      <c r="H16" s="16">
         <f>IF(H15&gt;0, VLOOKUP(H15-H$5-(INT($M15/9)+(MOD($M15,9)&gt;=H$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>0</v>
       </c>
-      <c r="I16" s="70">
+      <c r="I16" s="16">
         <f>IF(I15&gt;0, VLOOKUP(I15-I$5-(INT($M15/9)+(MOD($M15,9)&gt;=I$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="J16" s="70">
+      <c r="J16" s="16">
         <f>IF(J15&gt;0, VLOOKUP(J15-J$5-(INT($M15/9)+(MOD($M15,9)&gt;=J$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="K16" s="70">
+      <c r="K16" s="16">
         <f>IF(K15&gt;0, VLOOKUP(K15-K$5-(INT($M15/9)+(MOD($M15,9)&gt;=K$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="L16" s="71">
+      <c r="L16" s="17">
         <f t="shared" ref="L16" si="2">IF(SUM(C16:K16)&gt;0, SUM(C16:K16),"")</f>
         <v>13</v>
       </c>
@@ -9083,34 +9071,34 @@
         <v>15</v>
       </c>
       <c r="B17" s="12"/>
-      <c r="C17" s="68">
-        <v>5</v>
-      </c>
-      <c r="D17" s="68">
-        <v>6</v>
-      </c>
-      <c r="E17" s="68">
-        <v>5</v>
-      </c>
-      <c r="F17" s="68">
-        <v>6</v>
-      </c>
-      <c r="G17" s="68">
+      <c r="C17" s="12">
+        <v>5</v>
+      </c>
+      <c r="D17" s="12">
+        <v>6</v>
+      </c>
+      <c r="E17" s="12">
+        <v>5</v>
+      </c>
+      <c r="F17" s="12">
+        <v>6</v>
+      </c>
+      <c r="G17" s="12">
         <v>8</v>
       </c>
-      <c r="H17" s="68">
-        <v>5</v>
-      </c>
-      <c r="I17" s="68">
-        <v>6</v>
-      </c>
-      <c r="J17" s="68">
-        <v>6</v>
-      </c>
-      <c r="K17" s="68">
+      <c r="H17" s="12">
+        <v>5</v>
+      </c>
+      <c r="I17" s="12">
+        <v>6</v>
+      </c>
+      <c r="J17" s="12">
+        <v>6</v>
+      </c>
+      <c r="K17" s="12">
         <v>7</v>
       </c>
-      <c r="L17" s="69">
+      <c r="L17" s="13">
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
@@ -9137,43 +9125,43 @@
     <row r="18" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="15"/>
       <c r="B18" s="16"/>
-      <c r="C18" s="70">
+      <c r="C18" s="16">
         <f>IF(C17&gt;0, VLOOKUP(C17-C$5-(INT($M17/9)+(MOD($M17,9)&gt;=C$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="D18" s="70">
+      <c r="D18" s="16">
         <f>IF(D17&gt;0, VLOOKUP(D17-D$5-(INT($M17/9)+(MOD($M17,9)&gt;=D$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="E18" s="70">
+      <c r="E18" s="16">
         <f>IF(E17&gt;0, VLOOKUP(E17-E$5-(INT($M17/9)+(MOD($M17,9)&gt;=E$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="F18" s="70">
+      <c r="F18" s="16">
         <f>IF(F17&gt;0, VLOOKUP(F17-F$5-(INT($M17/9)+(MOD($M17,9)&gt;=F$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="G18" s="70">
+      <c r="G18" s="16">
         <f>IF(G17&gt;0, VLOOKUP(G17-G$5-(INT($M17/9)+(MOD($M17,9)&gt;=G$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>0</v>
       </c>
-      <c r="H18" s="70">
+      <c r="H18" s="16">
         <f>IF(H17&gt;0, VLOOKUP(H17-H$5-(INT($M17/9)+(MOD($M17,9)&gt;=H$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="I18" s="70">
+      <c r="I18" s="16">
         <f>IF(I17&gt;0, VLOOKUP(I17-I$5-(INT($M17/9)+(MOD($M17,9)&gt;=I$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="J18" s="70">
+      <c r="J18" s="16">
         <f>IF(J17&gt;0, VLOOKUP(J17-J$5-(INT($M17/9)+(MOD($M17,9)&gt;=J$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="K18" s="70">
+      <c r="K18" s="16">
         <f>IF(K17&gt;0, VLOOKUP(K17-K$5-(INT($M17/9)+(MOD($M17,9)&gt;=K$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="L18" s="71">
+      <c r="L18" s="17">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
@@ -9200,34 +9188,34 @@
         <v>16</v>
       </c>
       <c r="B19" s="12"/>
-      <c r="C19" s="68">
+      <c r="C19" s="12">
         <v>8</v>
       </c>
-      <c r="D19" s="68">
-        <v>5</v>
-      </c>
-      <c r="E19" s="68">
-        <v>5</v>
-      </c>
-      <c r="F19" s="68">
-        <v>3</v>
-      </c>
-      <c r="G19" s="68">
-        <v>6</v>
-      </c>
-      <c r="H19" s="68">
-        <v>5</v>
-      </c>
-      <c r="I19" s="68">
-        <v>6</v>
-      </c>
-      <c r="J19" s="68">
-        <v>6</v>
-      </c>
-      <c r="K19" s="68">
-        <v>6</v>
-      </c>
-      <c r="L19" s="69">
+      <c r="D19" s="12">
+        <v>5</v>
+      </c>
+      <c r="E19" s="12">
+        <v>5</v>
+      </c>
+      <c r="F19" s="12">
+        <v>3</v>
+      </c>
+      <c r="G19" s="12">
+        <v>6</v>
+      </c>
+      <c r="H19" s="12">
+        <v>5</v>
+      </c>
+      <c r="I19" s="12">
+        <v>6</v>
+      </c>
+      <c r="J19" s="12">
+        <v>6</v>
+      </c>
+      <c r="K19" s="12">
+        <v>6</v>
+      </c>
+      <c r="L19" s="13">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
@@ -9254,43 +9242,43 @@
     <row r="20" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="15"/>
       <c r="B20" s="16"/>
-      <c r="C20" s="70">
+      <c r="C20" s="16">
         <f>IF(C19&gt;0, VLOOKUP(C19-C$5-(INT($M19/9)+(MOD($M19,9)&gt;=C$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>0</v>
       </c>
-      <c r="D20" s="70">
+      <c r="D20" s="16">
         <f>IF(D19&gt;0, VLOOKUP(D19-D$5-(INT($M19/9)+(MOD($M19,9)&gt;=D$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>4</v>
       </c>
-      <c r="E20" s="70">
+      <c r="E20" s="16">
         <f>IF(E19&gt;0, VLOOKUP(E19-E$5-(INT($M19/9)+(MOD($M19,9)&gt;=E$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="F20" s="70">
+      <c r="F20" s="16">
         <f>IF(F19&gt;0, VLOOKUP(F19-F$5-(INT($M19/9)+(MOD($M19,9)&gt;=F$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="G20" s="70">
+      <c r="G20" s="16">
         <f>IF(G19&gt;0, VLOOKUP(G19-G$5-(INT($M19/9)+(MOD($M19,9)&gt;=G$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="H20" s="70">
+      <c r="H20" s="16">
         <f>IF(H19&gt;0, VLOOKUP(H19-H$5-(INT($M19/9)+(MOD($M19,9)&gt;=H$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="I20" s="70">
+      <c r="I20" s="16">
         <f>IF(I19&gt;0, VLOOKUP(I19-I$5-(INT($M19/9)+(MOD($M19,9)&gt;=I$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>0</v>
       </c>
-      <c r="J20" s="70">
+      <c r="J20" s="16">
         <f>IF(J19&gt;0, VLOOKUP(J19-J$5-(INT($M19/9)+(MOD($M19,9)&gt;=J$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="K20" s="70">
+      <c r="K20" s="16">
         <f>IF(K19&gt;0, VLOOKUP(K19-K$5-(INT($M19/9)+(MOD($M19,9)&gt;=K$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="L20" s="71">
+      <c r="L20" s="17">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
@@ -9317,34 +9305,34 @@
         <v>36</v>
       </c>
       <c r="B21" s="12"/>
-      <c r="C21" s="68">
-        <v>4</v>
-      </c>
-      <c r="D21" s="68">
-        <v>5</v>
-      </c>
-      <c r="E21" s="68">
-        <v>4</v>
-      </c>
-      <c r="F21" s="68">
-        <v>4</v>
-      </c>
-      <c r="G21" s="68">
-        <v>4</v>
-      </c>
-      <c r="H21" s="68">
-        <v>4</v>
-      </c>
-      <c r="I21" s="68">
-        <v>3</v>
-      </c>
-      <c r="J21" s="68">
-        <v>5</v>
-      </c>
-      <c r="K21" s="68">
-        <v>5</v>
-      </c>
-      <c r="L21" s="69">
+      <c r="C21" s="12">
+        <v>4</v>
+      </c>
+      <c r="D21" s="12">
+        <v>5</v>
+      </c>
+      <c r="E21" s="12">
+        <v>4</v>
+      </c>
+      <c r="F21" s="12">
+        <v>4</v>
+      </c>
+      <c r="G21" s="12">
+        <v>4</v>
+      </c>
+      <c r="H21" s="12">
+        <v>4</v>
+      </c>
+      <c r="I21" s="12">
+        <v>3</v>
+      </c>
+      <c r="J21" s="12">
+        <v>5</v>
+      </c>
+      <c r="K21" s="12">
+        <v>5</v>
+      </c>
+      <c r="L21" s="13">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
@@ -9371,43 +9359,43 @@
     <row r="22" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="15"/>
       <c r="B22" s="16"/>
-      <c r="C22" s="70">
+      <c r="C22" s="16">
         <f>IF(C21&gt;0, VLOOKUP(C21-C$5-(INT($M21/9)+(MOD($M21,9)&gt;=C$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="D22" s="70">
+      <c r="D22" s="16">
         <f>IF(D21&gt;0, VLOOKUP(D21-D$5-(INT($M21/9)+(MOD($M21,9)&gt;=D$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="E22" s="70">
+      <c r="E22" s="16">
         <f>IF(E21&gt;0, VLOOKUP(E21-E$5-(INT($M21/9)+(MOD($M21,9)&gt;=E$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="F22" s="70">
+      <c r="F22" s="16">
         <f>IF(F21&gt;0, VLOOKUP(F21-F$5-(INT($M21/9)+(MOD($M21,9)&gt;=F$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="G22" s="70">
+      <c r="G22" s="16">
         <f>IF(G21&gt;0, VLOOKUP(G21-G$5-(INT($M21/9)+(MOD($M21,9)&gt;=G$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="H22" s="70">
+      <c r="H22" s="16">
         <f>IF(H21&gt;0, VLOOKUP(H21-H$5-(INT($M21/9)+(MOD($M21,9)&gt;=H$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="I22" s="70">
+      <c r="I22" s="16">
         <f>IF(I21&gt;0, VLOOKUP(I21-I$5-(INT($M21/9)+(MOD($M21,9)&gt;=I$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="J22" s="70">
+      <c r="J22" s="16">
         <f>IF(J21&gt;0, VLOOKUP(J21-J$5-(INT($M21/9)+(MOD($M21,9)&gt;=J$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="K22" s="70">
+      <c r="K22" s="16">
         <f>IF(K21&gt;0, VLOOKUP(K21-K$5-(INT($M21/9)+(MOD($M21,9)&gt;=K$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="L22" s="71">
+      <c r="L22" s="17">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
@@ -9434,34 +9422,34 @@
         <v>11</v>
       </c>
       <c r="B23" s="12"/>
-      <c r="C23" s="68">
-        <v>5</v>
-      </c>
-      <c r="D23" s="68">
-        <v>5</v>
-      </c>
-      <c r="E23" s="68">
-        <v>5</v>
-      </c>
-      <c r="F23" s="68">
-        <v>4</v>
-      </c>
-      <c r="G23" s="68">
-        <v>4</v>
-      </c>
-      <c r="H23" s="68">
-        <v>4</v>
-      </c>
-      <c r="I23" s="68">
-        <v>4</v>
-      </c>
-      <c r="J23" s="68">
-        <v>4</v>
-      </c>
-      <c r="K23" s="68">
-        <v>6</v>
-      </c>
-      <c r="L23" s="69">
+      <c r="C23" s="12">
+        <v>5</v>
+      </c>
+      <c r="D23" s="12">
+        <v>5</v>
+      </c>
+      <c r="E23" s="12">
+        <v>5</v>
+      </c>
+      <c r="F23" s="12">
+        <v>4</v>
+      </c>
+      <c r="G23" s="12">
+        <v>4</v>
+      </c>
+      <c r="H23" s="12">
+        <v>4</v>
+      </c>
+      <c r="I23" s="12">
+        <v>4</v>
+      </c>
+      <c r="J23" s="12">
+        <v>4</v>
+      </c>
+      <c r="K23" s="12">
+        <v>6</v>
+      </c>
+      <c r="L23" s="13">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
@@ -9488,43 +9476,43 @@
     <row r="24" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="15"/>
       <c r="B24" s="16"/>
-      <c r="C24" s="70">
+      <c r="C24" s="16">
         <f>IF(C23&gt;0, VLOOKUP(C23-C$5-(INT($M23/9)+(MOD($M23,9)&gt;=C$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="D24" s="70">
+      <c r="D24" s="16">
         <f>IF(D23&gt;0, VLOOKUP(D23-D$5-(INT($M23/9)+(MOD($M23,9)&gt;=D$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="E24" s="70">
+      <c r="E24" s="16">
         <f>IF(E23&gt;0, VLOOKUP(E23-E$5-(INT($M23/9)+(MOD($M23,9)&gt;=E$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="F24" s="70">
+      <c r="F24" s="16">
         <f>IF(F23&gt;0, VLOOKUP(F23-F$5-(INT($M23/9)+(MOD($M23,9)&gt;=F$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="G24" s="70">
+      <c r="G24" s="16">
         <f>IF(G23&gt;0, VLOOKUP(G23-G$5-(INT($M23/9)+(MOD($M23,9)&gt;=G$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="H24" s="70">
+      <c r="H24" s="16">
         <f>IF(H23&gt;0, VLOOKUP(H23-H$5-(INT($M23/9)+(MOD($M23,9)&gt;=H$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="I24" s="70">
+      <c r="I24" s="16">
         <f>IF(I23&gt;0, VLOOKUP(I23-I$5-(INT($M23/9)+(MOD($M23,9)&gt;=I$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="J24" s="70">
+      <c r="J24" s="16">
         <f>IF(J23&gt;0, VLOOKUP(J23-J$5-(INT($M23/9)+(MOD($M23,9)&gt;=J$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="K24" s="70">
+      <c r="K24" s="16">
         <f>IF(K23&gt;0, VLOOKUP(K23-K$5-(INT($M23/9)+(MOD($M23,9)&gt;=K$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="L24" s="71">
+      <c r="L24" s="17">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
@@ -9551,34 +9539,34 @@
         <v>28</v>
       </c>
       <c r="B25" s="12"/>
-      <c r="C25" s="68">
-        <v>6</v>
-      </c>
-      <c r="D25" s="68">
+      <c r="C25" s="12">
+        <v>6</v>
+      </c>
+      <c r="D25" s="12">
         <v>10</v>
       </c>
-      <c r="E25" s="68">
+      <c r="E25" s="12">
         <v>8</v>
       </c>
-      <c r="F25" s="68">
-        <v>6</v>
-      </c>
-      <c r="G25" s="68">
+      <c r="F25" s="12">
+        <v>6</v>
+      </c>
+      <c r="G25" s="12">
         <v>8</v>
       </c>
-      <c r="H25" s="68">
+      <c r="H25" s="12">
         <v>8</v>
       </c>
-      <c r="I25" s="68">
-        <v>6</v>
-      </c>
-      <c r="J25" s="68">
+      <c r="I25" s="12">
+        <v>6</v>
+      </c>
+      <c r="J25" s="12">
         <v>8</v>
       </c>
-      <c r="K25" s="68">
+      <c r="K25" s="12">
         <v>10</v>
       </c>
-      <c r="L25" s="69">
+      <c r="L25" s="13">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
@@ -9605,43 +9593,43 @@
     <row r="26" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="15"/>
       <c r="B26" s="16"/>
-      <c r="C26" s="70">
+      <c r="C26" s="16">
         <f>IF(C25&gt;0, VLOOKUP(C25-C$5-(INT($M25/9)+(MOD($M25,9)&gt;=C$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="D26" s="70">
+      <c r="D26" s="16">
         <f>IF(D25&gt;0, VLOOKUP(D25-D$5-(INT($M25/9)+(MOD($M25,9)&gt;=D$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>0</v>
       </c>
-      <c r="E26" s="70">
+      <c r="E26" s="16">
         <f>IF(E25&gt;0, VLOOKUP(E25-E$5-(INT($M25/9)+(MOD($M25,9)&gt;=E$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="F26" s="70">
+      <c r="F26" s="16">
         <f>IF(F25&gt;0, VLOOKUP(F25-F$5-(INT($M25/9)+(MOD($M25,9)&gt;=F$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="G26" s="70">
+      <c r="G26" s="16">
         <f>IF(G25&gt;0, VLOOKUP(G25-G$5-(INT($M25/9)+(MOD($M25,9)&gt;=G$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>0</v>
       </c>
-      <c r="H26" s="70">
+      <c r="H26" s="16">
         <f>IF(H25&gt;0, VLOOKUP(H25-H$5-(INT($M25/9)+(MOD($M25,9)&gt;=H$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>0</v>
       </c>
-      <c r="I26" s="70">
+      <c r="I26" s="16">
         <f>IF(I25&gt;0, VLOOKUP(I25-I$5-(INT($M25/9)+(MOD($M25,9)&gt;=I$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="J26" s="70">
+      <c r="J26" s="16">
         <f>IF(J25&gt;0, VLOOKUP(J25-J$5-(INT($M25/9)+(MOD($M25,9)&gt;=J$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>0</v>
       </c>
-      <c r="K26" s="70">
+      <c r="K26" s="16">
         <f>IF(K25&gt;0, VLOOKUP(K25-K$5-(INT($M25/9)+(MOD($M25,9)&gt;=K$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>0</v>
       </c>
-      <c r="L26" s="71">
+      <c r="L26" s="17">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -9668,34 +9656,34 @@
         <v>35</v>
       </c>
       <c r="B27" s="12"/>
-      <c r="C27" s="68">
+      <c r="C27" s="12">
         <v>8</v>
       </c>
-      <c r="D27" s="68">
-        <v>6</v>
-      </c>
-      <c r="E27" s="68">
-        <v>5</v>
-      </c>
-      <c r="F27" s="68">
-        <v>6</v>
-      </c>
-      <c r="G27" s="68">
-        <v>6</v>
-      </c>
-      <c r="H27" s="68">
-        <v>5</v>
-      </c>
-      <c r="I27" s="68">
-        <v>4</v>
-      </c>
-      <c r="J27" s="68">
-        <v>6</v>
-      </c>
-      <c r="K27" s="68">
-        <v>6</v>
-      </c>
-      <c r="L27" s="69">
+      <c r="D27" s="12">
+        <v>6</v>
+      </c>
+      <c r="E27" s="12">
+        <v>5</v>
+      </c>
+      <c r="F27" s="12">
+        <v>6</v>
+      </c>
+      <c r="G27" s="12">
+        <v>6</v>
+      </c>
+      <c r="H27" s="12">
+        <v>5</v>
+      </c>
+      <c r="I27" s="12">
+        <v>4</v>
+      </c>
+      <c r="J27" s="12">
+        <v>6</v>
+      </c>
+      <c r="K27" s="12">
+        <v>6</v>
+      </c>
+      <c r="L27" s="13">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
@@ -9722,43 +9710,43 @@
     <row r="28" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="15"/>
       <c r="B28" s="16"/>
-      <c r="C28" s="70">
+      <c r="C28" s="16">
         <f>IF(C27&gt;0, VLOOKUP(C27-C$5-(INT($M27/9)+(MOD($M27,9)&gt;=C$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>0</v>
       </c>
-      <c r="D28" s="70">
+      <c r="D28" s="16">
         <f>IF(D27&gt;0, VLOOKUP(D27-D$5-(INT($M27/9)+(MOD($M27,9)&gt;=D$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="E28" s="70">
+      <c r="E28" s="16">
         <f>IF(E27&gt;0, VLOOKUP(E27-E$5-(INT($M27/9)+(MOD($M27,9)&gt;=E$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="F28" s="70">
+      <c r="F28" s="16">
         <f>IF(F27&gt;0, VLOOKUP(F27-F$5-(INT($M27/9)+(MOD($M27,9)&gt;=F$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>0</v>
       </c>
-      <c r="G28" s="70">
+      <c r="G28" s="16">
         <f>IF(G27&gt;0, VLOOKUP(G27-G$5-(INT($M27/9)+(MOD($M27,9)&gt;=G$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="H28" s="70">
+      <c r="H28" s="16">
         <f>IF(H27&gt;0, VLOOKUP(H27-H$5-(INT($M27/9)+(MOD($M27,9)&gt;=H$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="I28" s="70">
+      <c r="I28" s="16">
         <f>IF(I27&gt;0, VLOOKUP(I27-I$5-(INT($M27/9)+(MOD($M27,9)&gt;=I$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="J28" s="70">
+      <c r="J28" s="16">
         <f>IF(J27&gt;0, VLOOKUP(J27-J$5-(INT($M27/9)+(MOD($M27,9)&gt;=J$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="K28" s="70">
+      <c r="K28" s="16">
         <f>IF(K27&gt;0, VLOOKUP(K27-K$5-(INT($M27/9)+(MOD($M27,9)&gt;=K$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="L28" s="71">
+      <c r="L28" s="17">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
@@ -9785,34 +9773,34 @@
         <v>37</v>
       </c>
       <c r="B29" s="12"/>
-      <c r="C29" s="68">
-        <v>5</v>
-      </c>
-      <c r="D29" s="68">
-        <v>6</v>
-      </c>
-      <c r="E29" s="68">
-        <v>5</v>
-      </c>
-      <c r="F29" s="68">
-        <v>5</v>
-      </c>
-      <c r="G29" s="68">
-        <v>5</v>
-      </c>
-      <c r="H29" s="68">
-        <v>5</v>
-      </c>
-      <c r="I29" s="68">
-        <v>5</v>
-      </c>
-      <c r="J29" s="68">
+      <c r="C29" s="12">
+        <v>5</v>
+      </c>
+      <c r="D29" s="12">
+        <v>6</v>
+      </c>
+      <c r="E29" s="12">
+        <v>5</v>
+      </c>
+      <c r="F29" s="12">
+        <v>5</v>
+      </c>
+      <c r="G29" s="12">
+        <v>5</v>
+      </c>
+      <c r="H29" s="12">
+        <v>5</v>
+      </c>
+      <c r="I29" s="12">
+        <v>5</v>
+      </c>
+      <c r="J29" s="12">
         <v>7</v>
       </c>
-      <c r="K29" s="68">
+      <c r="K29" s="12">
         <v>7</v>
       </c>
-      <c r="L29" s="69">
+      <c r="L29" s="13">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
@@ -9839,43 +9827,43 @@
     <row r="30" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="15"/>
       <c r="B30" s="16"/>
-      <c r="C30" s="70">
+      <c r="C30" s="16">
         <f>IF(C29&gt;0, VLOOKUP(C29-C$5-(INT($M29/9)+(MOD($M29,9)&gt;=C$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="D30" s="70">
+      <c r="D30" s="16">
         <f>IF(D29&gt;0, VLOOKUP(D29-D$5-(INT($M29/9)+(MOD($M29,9)&gt;=D$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="E30" s="70">
+      <c r="E30" s="16">
         <f>IF(E29&gt;0, VLOOKUP(E29-E$5-(INT($M29/9)+(MOD($M29,9)&gt;=E$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="F30" s="70">
+      <c r="F30" s="16">
         <f>IF(F29&gt;0, VLOOKUP(F29-F$5-(INT($M29/9)+(MOD($M29,9)&gt;=F$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="G30" s="70">
+      <c r="G30" s="16">
         <f>IF(G29&gt;0, VLOOKUP(G29-G$5-(INT($M29/9)+(MOD($M29,9)&gt;=G$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
-      <c r="H30" s="70">
+      <c r="H30" s="16">
         <f>IF(H29&gt;0, VLOOKUP(H29-H$5-(INT($M29/9)+(MOD($M29,9)&gt;=H$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="I30" s="70">
+      <c r="I30" s="16">
         <f>IF(I29&gt;0, VLOOKUP(I29-I$5-(INT($M29/9)+(MOD($M29,9)&gt;=I$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="J30" s="70">
+      <c r="J30" s="16">
         <f>IF(J29&gt;0, VLOOKUP(J29-J$5-(INT($M29/9)+(MOD($M29,9)&gt;=J$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>0</v>
       </c>
-      <c r="K30" s="70">
+      <c r="K30" s="16">
         <f>IF(K29&gt;0, VLOOKUP(K29-K$5-(INT($M29/9)+(MOD($M29,9)&gt;=K$6)), '[2]Point System'!$A$4:$B$15, 2),"")</f>
         <v>2</v>
       </c>
-      <c r="L30" s="71">
+      <c r="L30" s="17">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>

</xml_diff>